<commit_message>
Updated PFlow dummy gen
</commit_message>
<xml_diff>
--- a/PFlow_2035/pp_PFlow_2035.xlsx
+++ b/PFlow_2035/pp_PFlow_2035.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piete\Documents\pieter\school\studie\Master\THESIS\CODE\HPvanRhee_MScThesis_Documentation\Modeling_Documentation\pp_andes_2035\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piete\Documents\pieter\school\studie\Master\THESIS\CODE\HPvanRhee_MScThesis_Documentation\PFlow_2035\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEA5D45-77DC-4464-84AB-C08F8588AB80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A22782-D5BE-41B9-B67F-372DB5E8A892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25815" yWindow="2580" windowWidth="21600" windowHeight="11295" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bus" sheetId="1" r:id="rId1"/>
@@ -1590,7 +1590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1616,10 +1616,11 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -3343,7 +3344,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{839BCD30-A54C-4CD0-B058-799BD1C0F64B}">
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -4469,7 +4470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -4504,7 +4505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -4539,7 +4540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -4574,7 +4575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -4608,8 +4609,11 @@
       <c r="L36" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
+      <c r="P36" s="20"/>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -4620,10 +4624,11 @@
         <v>38</v>
       </c>
       <c r="D37" s="16">
-        <v>599.25759999999991</v>
+        <v>979.25759999999991</v>
       </c>
       <c r="E37" s="16">
-        <v>196.96644802763311</v>
+        <f>TAN(ACOS(0.95))*D37</f>
+        <v>321.86640799560115</v>
       </c>
       <c r="F37">
         <v>0</v>
@@ -4643,9 +4648,11 @@
       <c r="L37" t="b">
         <v>0</v>
       </c>
-      <c r="O37" s="17"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N37" s="20"/>
+      <c r="O37" s="21"/>
+      <c r="P37" s="20"/>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -4656,10 +4663,11 @@
         <v>39</v>
       </c>
       <c r="D38" s="16">
-        <v>599.25759999999991</v>
+        <v>979.25759999999991</v>
       </c>
       <c r="E38" s="16">
-        <v>196.96644802763311</v>
+        <f t="shared" ref="E38:E46" si="0">TAN(ACOS(0.95))*D38</f>
+        <v>321.86640799560115</v>
       </c>
       <c r="F38">
         <v>0</v>
@@ -4679,9 +4687,11 @@
       <c r="L38" t="b">
         <v>0</v>
       </c>
-      <c r="O38" s="17"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N38" s="20"/>
+      <c r="O38" s="21"/>
+      <c r="P38" s="20"/>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -4692,10 +4702,11 @@
         <v>41</v>
       </c>
       <c r="D39" s="16">
-        <v>599.25759999999991</v>
+        <v>979.25759999999991</v>
       </c>
       <c r="E39" s="16">
-        <v>196.96644802763311</v>
+        <f t="shared" si="0"/>
+        <v>321.86640799560115</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -4715,9 +4726,11 @@
       <c r="L39" t="b">
         <v>0</v>
       </c>
-      <c r="O39" s="17"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N39" s="20"/>
+      <c r="O39" s="21"/>
+      <c r="P39" s="20"/>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -4728,10 +4741,11 @@
         <v>42</v>
       </c>
       <c r="D40" s="16">
-        <v>599.25759999999991</v>
+        <v>979.25759999999991</v>
       </c>
       <c r="E40" s="16">
-        <v>196.96644802763311</v>
+        <f t="shared" si="0"/>
+        <v>321.86640799560115</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -4751,9 +4765,11 @@
       <c r="L40" t="b">
         <v>0</v>
       </c>
-      <c r="O40" s="17"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N40" s="20"/>
+      <c r="O40" s="21"/>
+      <c r="P40" s="20"/>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -4764,10 +4780,11 @@
         <v>43</v>
       </c>
       <c r="D41" s="16">
-        <v>522.06799999999998</v>
+        <v>782.06799999999998</v>
       </c>
       <c r="E41" s="16">
-        <v>171.59545342251874</v>
+        <f t="shared" si="0"/>
+        <v>257.05332076902317</v>
       </c>
       <c r="F41">
         <v>0</v>
@@ -4787,9 +4804,11 @@
       <c r="L41" t="b">
         <v>0</v>
       </c>
-      <c r="O41" s="17"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N41" s="20"/>
+      <c r="O41" s="21"/>
+      <c r="P41" s="20"/>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -4800,10 +4819,11 @@
         <v>44</v>
       </c>
       <c r="D42" s="16">
-        <v>422.06799999999998</v>
+        <v>782.06799999999998</v>
       </c>
       <c r="E42" s="16">
-        <v>138.72704290463244</v>
+        <f t="shared" si="0"/>
+        <v>257.05332076902317</v>
       </c>
       <c r="F42">
         <v>0</v>
@@ -4823,9 +4843,11 @@
       <c r="L42" t="b">
         <v>0</v>
       </c>
-      <c r="O42" s="17"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N42" s="20"/>
+      <c r="O42" s="21"/>
+      <c r="P42" s="20"/>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -4836,10 +4858,11 @@
         <v>35</v>
       </c>
       <c r="D43" s="16">
-        <v>100</v>
+        <v>3580</v>
       </c>
       <c r="E43" s="16">
-        <v>32.868410517886325</v>
+        <f t="shared" si="0"/>
+        <v>1176.6890965403302</v>
       </c>
       <c r="F43">
         <v>0</v>
@@ -4859,8 +4882,11 @@
       <c r="L43" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N43" s="20"/>
+      <c r="O43" s="20"/>
+      <c r="P43" s="20"/>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -4871,10 +4897,11 @@
         <v>36</v>
       </c>
       <c r="D44" s="16">
-        <v>203.98</v>
+        <v>343.97999999999996</v>
       </c>
       <c r="E44" s="16">
-        <v>67.044983774384519</v>
+        <f t="shared" si="0"/>
+        <v>113.06075849942535</v>
       </c>
       <c r="F44">
         <v>0</v>
@@ -4894,9 +4921,11 @@
       <c r="L44" t="b">
         <v>0</v>
       </c>
-      <c r="O44" s="17"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N44" s="20"/>
+      <c r="O44" s="21"/>
+      <c r="P44" s="20"/>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -4907,10 +4936,11 @@
         <v>37</v>
       </c>
       <c r="D45" s="16">
-        <v>100</v>
+        <v>4100</v>
       </c>
       <c r="E45" s="16">
-        <v>32.868410517886325</v>
+        <f t="shared" si="0"/>
+        <v>1347.6048312333392</v>
       </c>
       <c r="F45">
         <v>0</v>
@@ -4930,8 +4960,11 @@
       <c r="L45" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N45" s="20"/>
+      <c r="O45" s="20"/>
+      <c r="P45" s="20"/>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -4942,10 +4975,11 @@
         <v>40</v>
       </c>
       <c r="D46" s="16">
-        <v>599.25759999999991</v>
+        <v>979.25759999999991</v>
       </c>
       <c r="E46" s="16">
-        <v>196.96644802763311</v>
+        <f t="shared" si="0"/>
+        <v>321.86640799560115</v>
       </c>
       <c r="F46">
         <v>0</v>
@@ -4965,30 +4999,43 @@
       <c r="L46" t="b">
         <v>0</v>
       </c>
-      <c r="O46" s="17"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N46" s="20"/>
+      <c r="O46" s="21"/>
+      <c r="P46" s="20"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N47" s="20"/>
+      <c r="O47" s="20"/>
+      <c r="P47" s="20"/>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="N48" s="20"/>
+      <c r="O48" s="20"/>
+      <c r="P48" s="20"/>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="N49" s="20"/>
+      <c r="O49" s="20"/>
+      <c r="P49" s="20"/>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="9"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="9"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="9"/>
     </row>
   </sheetData>
@@ -5063,8 +5110,8 @@
         <v>38</v>
       </c>
       <c r="D2" s="16">
-        <f>0.05*2000</f>
-        <v>100</v>
+        <f>0.24*2000</f>
+        <v>480</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -5094,10 +5141,11 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>-1972</v>
+        <f>-P2</f>
+        <v>-2340</v>
       </c>
       <c r="P2">
-        <v>1972</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -5111,8 +5159,8 @@
         <v>39</v>
       </c>
       <c r="D3" s="16">
-        <f t="shared" ref="D3:D9" si="0">0.05*2000</f>
-        <v>100</v>
+        <f t="shared" ref="D3:D5" si="0">0.24*2000</f>
+        <v>480</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -5142,10 +5190,11 @@
         <v>1</v>
       </c>
       <c r="O3">
-        <v>-1972</v>
+        <f t="shared" ref="O3:O10" si="1">-P3</f>
+        <v>-2340</v>
       </c>
       <c r="P3">
-        <v>1972</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -5160,7 +5209,7 @@
       </c>
       <c r="D4" s="16">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>480</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -5190,10 +5239,11 @@
         <v>1</v>
       </c>
       <c r="O4">
-        <v>-986</v>
+        <f t="shared" si="1"/>
+        <v>-2340</v>
       </c>
       <c r="P4">
-        <v>986</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -5208,7 +5258,7 @@
       </c>
       <c r="D5" s="16">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>480</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -5238,10 +5288,11 @@
         <v>1</v>
       </c>
       <c r="O5">
-        <v>-986</v>
+        <f t="shared" si="1"/>
+        <v>-2340</v>
       </c>
       <c r="P5">
-        <v>986</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -5255,8 +5306,8 @@
         <v>43</v>
       </c>
       <c r="D6" s="16">
-        <f t="shared" si="0"/>
-        <v>100</v>
+        <f>0.18*2000</f>
+        <v>360</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -5286,10 +5337,11 @@
         <v>1</v>
       </c>
       <c r="O6">
-        <v>-1128</v>
+        <f t="shared" si="1"/>
+        <v>-1200</v>
       </c>
       <c r="P6">
-        <v>1128</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -5303,8 +5355,8 @@
         <v>44</v>
       </c>
       <c r="D7" s="16">
-        <f t="shared" si="0"/>
-        <v>100</v>
+        <f>0.18*2000</f>
+        <v>360</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -5334,10 +5386,11 @@
         <v>1</v>
       </c>
       <c r="O7">
-        <v>-1128</v>
+        <f t="shared" si="1"/>
+        <v>-1200</v>
       </c>
       <c r="P7">
-        <v>1128</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -5351,8 +5404,8 @@
         <v>35</v>
       </c>
       <c r="D8" s="16">
-        <f>0.050432*2000</f>
-        <v>100.86399999999999</v>
+        <f>(0.050432*2000) - 100 + (2000*1.79)</f>
+        <v>3580.864</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -5382,10 +5435,11 @@
         <v>1</v>
       </c>
       <c r="O8">
-        <v>-1000</v>
+        <f t="shared" si="1"/>
+        <v>-10800</v>
       </c>
       <c r="P8">
-        <v>1000</v>
+        <v>10800</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -5399,8 +5453,8 @@
         <v>36</v>
       </c>
       <c r="D9" s="16">
-        <f t="shared" si="0"/>
-        <v>100</v>
+        <f>0.12*2000</f>
+        <v>240</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -5430,10 +5484,11 @@
         <v>1</v>
       </c>
       <c r="O9">
-        <v>-700</v>
+        <f t="shared" si="1"/>
+        <v>-1200</v>
       </c>
       <c r="P9">
-        <v>700</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -5447,8 +5502,8 @@
         <v>37</v>
       </c>
       <c r="D10" s="16">
-        <f>0.24611*2000</f>
-        <v>492.21999999999997</v>
+        <f>(0.24611-0.05+2.05)*2000</f>
+        <v>4492.2199999999993</v>
       </c>
       <c r="E10" s="3">
         <v>1</v>
@@ -5478,11 +5533,12 @@
       <c r="N10" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="O10" s="3">
-        <v>-700</v>
+      <c r="O10">
+        <f t="shared" si="1"/>
+        <v>-11100</v>
       </c>
       <c r="P10" s="3">
-        <v>700</v>
+        <v>11100</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -5546,18 +5602,18 @@
         <v>28</v>
       </c>
       <c r="D12">
-        <f t="shared" ref="D12:D75" si="1">0.6*P12</f>
+        <f t="shared" ref="D12:D75" si="2">0.6*P12</f>
         <v>75</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
       <c r="G12">
-        <f t="shared" ref="G12:G75" si="2">-H12</f>
+        <f t="shared" ref="G12:G75" si="3">-H12</f>
         <v>-41.25</v>
       </c>
       <c r="H12">
-        <f t="shared" ref="H12:H75" si="3">0.33*P12</f>
+        <f t="shared" ref="H12:H75" si="4">0.33*P12</f>
         <v>41.25</v>
       </c>
       <c r="I12">
@@ -5596,18 +5652,18 @@
         <v>29</v>
       </c>
       <c r="D13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.2</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
       <c r="G13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-2.31</v>
       </c>
       <c r="H13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.31</v>
       </c>
       <c r="I13">
@@ -5646,18 +5702,18 @@
         <v>12</v>
       </c>
       <c r="D14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>22.8</v>
       </c>
       <c r="E14">
         <v>1</v>
       </c>
       <c r="G14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-12.540000000000001</v>
       </c>
       <c r="H14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>12.540000000000001</v>
       </c>
       <c r="I14">
@@ -5695,7 +5751,7 @@
       <c r="C15">
         <v>11</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="18">
         <f>0.98*P15</f>
         <v>475.3</v>
       </c>
@@ -5703,11 +5759,11 @@
         <v>1</v>
       </c>
       <c r="G15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-160.05000000000001</v>
       </c>
       <c r="H15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>160.05000000000001</v>
       </c>
       <c r="I15">
@@ -5746,18 +5802,18 @@
         <v>9</v>
       </c>
       <c r="D16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>28.799999999999997</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
       <c r="G16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-15.84</v>
       </c>
       <c r="H16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>15.84</v>
       </c>
       <c r="I16">
@@ -5796,18 +5852,18 @@
         <v>11</v>
       </c>
       <c r="D17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>273</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="G17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-150.15</v>
       </c>
       <c r="H17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>150.15</v>
       </c>
       <c r="I17">
@@ -5846,18 +5902,18 @@
         <v>28</v>
       </c>
       <c r="D18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>506.4</v>
       </c>
       <c r="E18">
         <v>1</v>
       </c>
       <c r="G18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-278.52000000000004</v>
       </c>
       <c r="H18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>278.52000000000004</v>
       </c>
       <c r="I18">
@@ -5896,18 +5952,18 @@
         <v>3</v>
       </c>
       <c r="D19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>43.199999999999996</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="G19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-23.76</v>
       </c>
       <c r="H19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>23.76</v>
       </c>
       <c r="I19">
@@ -5946,18 +6002,18 @@
         <v>3</v>
       </c>
       <c r="D20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>43.199999999999996</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
       <c r="G20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-23.76</v>
       </c>
       <c r="H20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>23.76</v>
       </c>
       <c r="I20">
@@ -5996,18 +6052,18 @@
         <v>6</v>
       </c>
       <c r="D21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>78.599999999999994</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
       <c r="G21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-43.230000000000004</v>
       </c>
       <c r="H21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>43.230000000000004</v>
       </c>
       <c r="I21">
@@ -6046,18 +6102,18 @@
         <v>6</v>
       </c>
       <c r="D22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>215.4</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
       <c r="G22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-118.47</v>
       </c>
       <c r="H22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>118.47</v>
       </c>
       <c r="I22">
@@ -6096,18 +6152,18 @@
         <v>6</v>
       </c>
       <c r="D23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>215.4</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
       <c r="G23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-118.47</v>
       </c>
       <c r="H23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>118.47</v>
       </c>
       <c r="I23">
@@ -6146,18 +6202,18 @@
         <v>6</v>
       </c>
       <c r="D24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>216.6</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="G24">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-119.13000000000001</v>
       </c>
       <c r="H24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>119.13000000000001</v>
       </c>
       <c r="I24">
@@ -6196,18 +6252,18 @@
         <v>18</v>
       </c>
       <c r="D25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>215.4</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="G25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-118.47</v>
       </c>
       <c r="H25">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>118.47</v>
       </c>
       <c r="I25">
@@ -6246,18 +6302,18 @@
         <v>18</v>
       </c>
       <c r="D26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>216</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="G26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-118.80000000000001</v>
       </c>
       <c r="H26">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>118.80000000000001</v>
       </c>
       <c r="I26">
@@ -6296,18 +6352,18 @@
         <v>25</v>
       </c>
       <c r="D27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>255.6</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="G27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-140.58000000000001</v>
       </c>
       <c r="H27">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>140.58000000000001</v>
       </c>
       <c r="I27">
@@ -6346,18 +6402,18 @@
         <v>25</v>
       </c>
       <c r="D28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>249</v>
       </c>
       <c r="E28">
         <v>1</v>
       </c>
       <c r="G28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-136.95000000000002</v>
       </c>
       <c r="H28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>136.95000000000002</v>
       </c>
       <c r="I28">
@@ -6396,18 +6452,18 @@
         <v>13</v>
       </c>
       <c r="D29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>49.8</v>
       </c>
       <c r="E29">
         <v>1</v>
       </c>
       <c r="G29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-27.39</v>
       </c>
       <c r="H29">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>27.39</v>
       </c>
       <c r="I29">
@@ -6446,18 +6502,18 @@
         <v>33</v>
       </c>
       <c r="D30">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.2</v>
       </c>
       <c r="E30">
         <v>1</v>
       </c>
       <c r="G30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-36.96</v>
       </c>
       <c r="H30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>36.96</v>
       </c>
       <c r="I30">
@@ -6496,18 +6552,18 @@
         <v>24</v>
       </c>
       <c r="D31">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.399999999999999</v>
       </c>
       <c r="E31">
         <v>1</v>
       </c>
       <c r="G31">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-7.92</v>
       </c>
       <c r="H31">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7.92</v>
       </c>
       <c r="I31">
@@ -6546,18 +6602,18 @@
         <v>24</v>
       </c>
       <c r="D32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.399999999999999</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="G32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-7.92</v>
       </c>
       <c r="H32">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7.92</v>
       </c>
       <c r="I32">
@@ -6596,18 +6652,18 @@
         <v>24</v>
       </c>
       <c r="D33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>132</v>
       </c>
       <c r="E33">
         <v>1</v>
       </c>
       <c r="G33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-72.600000000000009</v>
       </c>
       <c r="H33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>72.600000000000009</v>
       </c>
       <c r="I33">
@@ -6646,18 +6702,18 @@
         <v>28</v>
       </c>
       <c r="D34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>47.4</v>
       </c>
       <c r="E34">
         <v>1</v>
       </c>
       <c r="G34">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-26.07</v>
       </c>
       <c r="H34">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>26.07</v>
       </c>
       <c r="I34">
@@ -6696,18 +6752,18 @@
         <v>11</v>
       </c>
       <c r="D35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>261</v>
       </c>
       <c r="E35">
         <v>1</v>
       </c>
       <c r="G35">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-143.55000000000001</v>
       </c>
       <c r="H35">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>143.55000000000001</v>
       </c>
       <c r="I35">
@@ -6746,18 +6802,18 @@
         <v>11</v>
       </c>
       <c r="D36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>261</v>
       </c>
       <c r="E36">
         <v>1</v>
       </c>
       <c r="G36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-143.55000000000001</v>
       </c>
       <c r="H36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>143.55000000000001</v>
       </c>
       <c r="I36">
@@ -6796,18 +6852,18 @@
         <v>22</v>
       </c>
       <c r="D37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>360</v>
       </c>
       <c r="E37">
         <v>1</v>
       </c>
       <c r="G37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-198</v>
       </c>
       <c r="H37">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>198</v>
       </c>
       <c r="I37">
@@ -6846,18 +6902,18 @@
         <v>23</v>
       </c>
       <c r="D38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36</v>
       </c>
       <c r="E38">
         <v>1</v>
       </c>
       <c r="G38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-19.8</v>
       </c>
       <c r="H38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>19.8</v>
       </c>
       <c r="I38">
@@ -6896,18 +6952,18 @@
         <v>8</v>
       </c>
       <c r="D39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>108</v>
       </c>
       <c r="E39">
         <v>1</v>
       </c>
       <c r="G39">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-59.400000000000006</v>
       </c>
       <c r="H39">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>59.400000000000006</v>
       </c>
       <c r="I39">
@@ -6946,18 +7002,18 @@
         <v>26</v>
       </c>
       <c r="D40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>384</v>
       </c>
       <c r="E40">
         <v>1</v>
       </c>
       <c r="G40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-211.20000000000002</v>
       </c>
       <c r="H40">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>211.20000000000002</v>
       </c>
       <c r="I40">
@@ -6996,18 +7052,18 @@
         <v>26</v>
       </c>
       <c r="D41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>765</v>
       </c>
       <c r="E41">
         <v>1</v>
       </c>
       <c r="G41">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-420.75</v>
       </c>
       <c r="H41">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>420.75</v>
       </c>
       <c r="I41">
@@ -7046,18 +7102,18 @@
         <v>8</v>
       </c>
       <c r="D42">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>210</v>
       </c>
       <c r="E42">
         <v>1</v>
       </c>
       <c r="G42">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-115.5</v>
       </c>
       <c r="H42">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>115.5</v>
       </c>
       <c r="I42">
@@ -7096,18 +7152,18 @@
         <v>9</v>
       </c>
       <c r="D43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>37.799999999999997</v>
       </c>
       <c r="E43">
         <v>1</v>
       </c>
       <c r="G43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20.790000000000003</v>
       </c>
       <c r="H43">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>20.790000000000003</v>
       </c>
       <c r="I43">
@@ -7146,18 +7202,18 @@
         <v>9</v>
       </c>
       <c r="D44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>37.799999999999997</v>
       </c>
       <c r="E44">
         <v>1</v>
       </c>
       <c r="G44">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20.790000000000003</v>
       </c>
       <c r="H44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>20.790000000000003</v>
       </c>
       <c r="I44">
@@ -7196,18 +7252,18 @@
         <v>26</v>
       </c>
       <c r="D45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>138</v>
       </c>
       <c r="E45">
         <v>1</v>
       </c>
       <c r="G45">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-75.900000000000006</v>
       </c>
       <c r="H45">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>75.900000000000006</v>
       </c>
       <c r="I45">
@@ -7246,18 +7302,18 @@
         <v>30</v>
       </c>
       <c r="D46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>19.8</v>
       </c>
       <c r="E46">
         <v>1</v>
       </c>
       <c r="G46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-10.89</v>
       </c>
       <c r="H46">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10.89</v>
       </c>
       <c r="I46">
@@ -7296,18 +7352,18 @@
         <v>16</v>
       </c>
       <c r="D47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="E47">
         <v>1</v>
       </c>
       <c r="G47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-8.25</v>
       </c>
       <c r="H47">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8.25</v>
       </c>
       <c r="I47">
@@ -7346,18 +7402,18 @@
         <v>22</v>
       </c>
       <c r="D48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>19.2</v>
       </c>
       <c r="E48">
         <v>1</v>
       </c>
       <c r="G48">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-10.56</v>
       </c>
       <c r="H48">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10.56</v>
       </c>
       <c r="I48">
@@ -7396,18 +7452,18 @@
         <v>2</v>
       </c>
       <c r="D49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>76.8</v>
       </c>
       <c r="E49">
         <v>1</v>
       </c>
       <c r="G49">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-42.24</v>
       </c>
       <c r="H49">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>42.24</v>
       </c>
       <c r="I49">
@@ -7446,18 +7502,18 @@
         <v>15</v>
       </c>
       <c r="D50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>37.199999999999996</v>
       </c>
       <c r="E50">
         <v>1</v>
       </c>
       <c r="G50">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-20.46</v>
       </c>
       <c r="H50">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>20.46</v>
       </c>
       <c r="I50">
@@ -7496,18 +7552,18 @@
         <v>15</v>
       </c>
       <c r="D51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>33</v>
       </c>
       <c r="E51">
         <v>1</v>
       </c>
       <c r="G51">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-18.150000000000002</v>
       </c>
       <c r="H51">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>18.150000000000002</v>
       </c>
       <c r="I51">
@@ -7546,18 +7602,18 @@
         <v>15</v>
       </c>
       <c r="D52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>149.4</v>
       </c>
       <c r="E52">
         <v>1</v>
       </c>
       <c r="G52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-82.17</v>
       </c>
       <c r="H52">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>82.17</v>
       </c>
       <c r="I52">
@@ -7596,18 +7652,18 @@
         <v>12</v>
       </c>
       <c r="D53">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>86.399999999999991</v>
       </c>
       <c r="E53">
         <v>1</v>
       </c>
       <c r="G53">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-47.52</v>
       </c>
       <c r="H53">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>47.52</v>
       </c>
       <c r="I53">
@@ -7646,18 +7702,18 @@
         <v>10</v>
       </c>
       <c r="D54">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>148.79999999999998</v>
       </c>
       <c r="E54">
         <v>1</v>
       </c>
       <c r="G54">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-81.84</v>
       </c>
       <c r="H54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>81.84</v>
       </c>
       <c r="I54">
@@ -7696,18 +7752,18 @@
         <v>10</v>
       </c>
       <c r="D55">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>61.8</v>
       </c>
       <c r="E55">
         <v>1</v>
       </c>
       <c r="G55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-33.99</v>
       </c>
       <c r="H55">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>33.99</v>
       </c>
       <c r="I55">
@@ -7746,18 +7802,18 @@
         <v>10</v>
       </c>
       <c r="D56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>135</v>
       </c>
       <c r="E56">
         <v>1</v>
       </c>
       <c r="G56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-74.25</v>
       </c>
       <c r="H56">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>74.25</v>
       </c>
       <c r="I56">
@@ -7796,18 +7852,18 @@
         <v>15</v>
       </c>
       <c r="D57">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>40.199999999999996</v>
       </c>
       <c r="E57">
         <v>1</v>
       </c>
       <c r="G57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-22.11</v>
       </c>
       <c r="H57">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>22.11</v>
       </c>
       <c r="I57">
@@ -7846,18 +7902,18 @@
         <v>12</v>
       </c>
       <c r="D58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>276</v>
       </c>
       <c r="E58">
         <v>1</v>
       </c>
       <c r="G58">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-151.80000000000001</v>
       </c>
       <c r="H58">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>151.80000000000001</v>
       </c>
       <c r="I58">
@@ -7896,18 +7952,18 @@
         <v>12</v>
       </c>
       <c r="D59">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>228</v>
       </c>
       <c r="E59">
         <v>1</v>
       </c>
       <c r="G59">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-125.4</v>
       </c>
       <c r="H59">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>125.4</v>
       </c>
       <c r="I59">
@@ -7946,18 +8002,18 @@
         <v>29</v>
       </c>
       <c r="D60">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>264</v>
       </c>
       <c r="E60">
         <v>1</v>
       </c>
       <c r="G60">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-145.20000000000002</v>
       </c>
       <c r="H60">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>145.20000000000002</v>
       </c>
       <c r="I60">
@@ -7996,18 +8052,18 @@
         <v>28</v>
       </c>
       <c r="D61">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>255.6</v>
       </c>
       <c r="E61">
         <v>1</v>
       </c>
       <c r="G61">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-140.58000000000001</v>
       </c>
       <c r="H61">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>140.58000000000001</v>
       </c>
       <c r="I61">
@@ -8046,18 +8102,18 @@
         <v>22</v>
       </c>
       <c r="D62">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>210.6</v>
       </c>
       <c r="E62">
         <v>1</v>
       </c>
       <c r="G62">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-115.83000000000001</v>
       </c>
       <c r="H62">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>115.83000000000001</v>
       </c>
       <c r="I62">
@@ -8096,18 +8152,18 @@
         <v>22</v>
       </c>
       <c r="D63">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>249</v>
       </c>
       <c r="E63">
         <v>1</v>
       </c>
       <c r="G63">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-136.95000000000002</v>
       </c>
       <c r="H63">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>136.95000000000002</v>
       </c>
       <c r="I63">
@@ -8146,18 +8202,18 @@
         <v>30</v>
       </c>
       <c r="D64">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.399999999999999</v>
       </c>
       <c r="E64">
         <v>1</v>
       </c>
       <c r="G64">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-7.92</v>
       </c>
       <c r="H64">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7.92</v>
       </c>
       <c r="I64">
@@ -8196,18 +8252,18 @@
         <v>21</v>
       </c>
       <c r="D65">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>262.2</v>
       </c>
       <c r="E65">
         <v>1</v>
       </c>
       <c r="G65">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-144.21</v>
       </c>
       <c r="H65">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>144.21</v>
       </c>
       <c r="I65">
@@ -8246,18 +8302,18 @@
         <v>21</v>
       </c>
       <c r="D66">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>262.2</v>
       </c>
       <c r="E66">
         <v>1</v>
       </c>
       <c r="G66">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-144.21</v>
       </c>
       <c r="H66">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>144.21</v>
       </c>
       <c r="I66">
@@ -8296,18 +8352,18 @@
         <v>21</v>
       </c>
       <c r="D67">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>262.2</v>
       </c>
       <c r="E67">
         <v>1</v>
       </c>
       <c r="G67">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-144.21</v>
       </c>
       <c r="H67">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>144.21</v>
       </c>
       <c r="I67">
@@ -8346,18 +8402,18 @@
         <v>15</v>
       </c>
       <c r="D68">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>261</v>
       </c>
       <c r="E68">
         <v>1</v>
       </c>
       <c r="G68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-143.55000000000001</v>
       </c>
       <c r="H68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>143.55000000000001</v>
       </c>
       <c r="I68">
@@ -8396,18 +8452,18 @@
         <v>22</v>
       </c>
       <c r="D69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="E69">
         <v>1</v>
       </c>
       <c r="G69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-39.6</v>
       </c>
       <c r="H69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>39.6</v>
       </c>
       <c r="I69">
@@ -8446,18 +8502,18 @@
         <v>22</v>
       </c>
       <c r="D70">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>21.599999999999998</v>
       </c>
       <c r="E70">
         <v>1</v>
       </c>
       <c r="G70">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-11.88</v>
       </c>
       <c r="H70">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>11.88</v>
       </c>
       <c r="I70">
@@ -8496,18 +8552,18 @@
         <v>23</v>
       </c>
       <c r="D71">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>13.799999999999999</v>
       </c>
       <c r="E71">
         <v>1</v>
       </c>
       <c r="G71">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-7.5900000000000007</v>
       </c>
       <c r="H71">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7.5900000000000007</v>
       </c>
       <c r="I71">
@@ -8546,18 +8602,18 @@
         <v>8</v>
       </c>
       <c r="D72">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="E72">
         <v>1</v>
       </c>
       <c r="G72">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-16.5</v>
       </c>
       <c r="H72">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>16.5</v>
       </c>
       <c r="I72">
@@ -8596,18 +8652,18 @@
         <v>51</v>
       </c>
       <c r="D73">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>73.2</v>
       </c>
       <c r="E73">
         <v>1</v>
       </c>
       <c r="G73">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-40.260000000000005</v>
       </c>
       <c r="H73">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>40.260000000000005</v>
       </c>
       <c r="I73">
@@ -8646,18 +8702,18 @@
         <v>17</v>
       </c>
       <c r="D74">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18.599999999999998</v>
       </c>
       <c r="E74">
         <v>1</v>
       </c>
       <c r="G74">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-10.23</v>
       </c>
       <c r="H74">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10.23</v>
       </c>
       <c r="I74">
@@ -8696,18 +8752,18 @@
         <v>23</v>
       </c>
       <c r="D75">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="E75">
         <v>1</v>
       </c>
       <c r="G75">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-16.5</v>
       </c>
       <c r="H75">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>16.5</v>
       </c>
       <c r="I75">
@@ -8746,18 +8802,18 @@
         <v>8</v>
       </c>
       <c r="D76">
-        <f t="shared" ref="D76:D82" si="4">0.6*P76</f>
+        <f t="shared" ref="D76:D82" si="5">0.6*P76</f>
         <v>21.599999999999998</v>
       </c>
       <c r="E76">
         <v>1</v>
       </c>
       <c r="G76">
-        <f t="shared" ref="G76:G82" si="5">-H76</f>
+        <f t="shared" ref="G76:G82" si="6">-H76</f>
         <v>-11.88</v>
       </c>
       <c r="H76">
-        <f t="shared" ref="H76:H82" si="6">0.33*P76</f>
+        <f t="shared" ref="H76:H82" si="7">0.33*P76</f>
         <v>11.88</v>
       </c>
       <c r="I76">
@@ -8796,18 +8852,18 @@
         <v>12</v>
       </c>
       <c r="D77">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>39</v>
       </c>
       <c r="E77">
         <v>1</v>
       </c>
       <c r="G77">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-21.45</v>
       </c>
       <c r="H77">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>21.45</v>
       </c>
       <c r="I77">
@@ -8846,18 +8902,18 @@
         <v>14</v>
       </c>
       <c r="D78">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>19.2</v>
       </c>
       <c r="E78">
         <v>1</v>
       </c>
       <c r="G78">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-10.56</v>
       </c>
       <c r="H78">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>10.56</v>
       </c>
       <c r="I78">
@@ -8896,18 +8952,18 @@
         <v>29</v>
       </c>
       <c r="D79">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>90</v>
       </c>
       <c r="E79">
         <v>1</v>
       </c>
       <c r="G79">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-49.5</v>
       </c>
       <c r="H79">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>49.5</v>
       </c>
       <c r="I79">
@@ -8946,18 +9002,18 @@
         <v>51</v>
       </c>
       <c r="D80">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>36</v>
       </c>
       <c r="E80">
         <v>1</v>
       </c>
       <c r="G80">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-19.8</v>
       </c>
       <c r="H80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>19.8</v>
       </c>
       <c r="I80">
@@ -8996,18 +9052,18 @@
         <v>50</v>
       </c>
       <c r="D81">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>19.2</v>
       </c>
       <c r="E81">
         <v>1</v>
       </c>
       <c r="G81">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-10.56</v>
       </c>
       <c r="H81">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>10.56</v>
       </c>
       <c r="I81">
@@ -9046,18 +9102,18 @@
         <v>48</v>
       </c>
       <c r="D82">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>30</v>
       </c>
       <c r="E82">
         <v>1</v>
       </c>
       <c r="G82">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-16.5</v>
       </c>
       <c r="H82">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>16.5</v>
       </c>
       <c r="I82">
@@ -9095,7 +9151,7 @@
       <c r="C83">
         <v>21</v>
       </c>
-      <c r="D83" s="18">
+      <c r="D83" s="17">
         <f>0.35*gen!P83</f>
         <v>210</v>
       </c>
@@ -9103,7 +9159,7 @@
         <v>1</v>
       </c>
       <c r="G83">
-        <f t="shared" ref="G83:G114" si="7">-H83</f>
+        <f t="shared" ref="G83:G114" si="8">-H83</f>
         <v>-198</v>
       </c>
       <c r="H83">
@@ -9145,7 +9201,7 @@
       <c r="C84">
         <v>13</v>
       </c>
-      <c r="D84" s="18">
+      <c r="D84" s="17">
         <f>0.35*gen!P84</f>
         <v>45.15</v>
       </c>
@@ -9153,7 +9209,7 @@
         <v>1</v>
       </c>
       <c r="G84">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-42.57</v>
       </c>
       <c r="H84">
@@ -9195,7 +9251,7 @@
       <c r="C85">
         <v>12</v>
       </c>
-      <c r="D85" s="18">
+      <c r="D85" s="17">
         <f>0.35*gen!P85</f>
         <v>42</v>
       </c>
@@ -9203,7 +9259,7 @@
         <v>1</v>
       </c>
       <c r="G85">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-39.6</v>
       </c>
       <c r="H85">
@@ -9245,7 +9301,7 @@
       <c r="C86">
         <v>12</v>
       </c>
-      <c r="D86" s="18">
+      <c r="D86" s="17">
         <f>0.35*gen!P86</f>
         <v>37.799999999999997</v>
       </c>
@@ -9253,7 +9309,7 @@
         <v>1</v>
       </c>
       <c r="G86">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-35.64</v>
       </c>
       <c r="H86">
@@ -9295,7 +9351,7 @@
       <c r="C87">
         <v>15</v>
       </c>
-      <c r="D87" s="18">
+      <c r="D87" s="17">
         <f>0.35*gen!P87</f>
         <v>42.699999999999996</v>
       </c>
@@ -9303,7 +9359,7 @@
         <v>1</v>
       </c>
       <c r="G87">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-40.260000000000005</v>
       </c>
       <c r="H87">
@@ -9345,7 +9401,7 @@
       <c r="C88">
         <v>6</v>
       </c>
-      <c r="D88" s="18">
+      <c r="D88" s="17">
         <f>0.35*gen!P88</f>
         <v>59.849999999999994</v>
       </c>
@@ -9353,7 +9409,7 @@
         <v>1</v>
       </c>
       <c r="G88">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-56.43</v>
       </c>
       <c r="H88">
@@ -9395,7 +9451,7 @@
       <c r="C89">
         <v>5</v>
       </c>
-      <c r="D89" s="18">
+      <c r="D89" s="17">
         <f>0.35*gen!P89</f>
         <v>50.4</v>
       </c>
@@ -9403,7 +9459,7 @@
         <v>1</v>
       </c>
       <c r="G89">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-47.52</v>
       </c>
       <c r="H89">
@@ -9445,7 +9501,7 @@
       <c r="C90">
         <v>5</v>
       </c>
-      <c r="D90" s="18">
+      <c r="D90" s="17">
         <f>0.35*gen!P90</f>
         <v>99.75</v>
       </c>
@@ -9453,7 +9509,7 @@
         <v>1</v>
       </c>
       <c r="G90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-94.050000000000011</v>
       </c>
       <c r="H90">
@@ -9495,7 +9551,7 @@
       <c r="C91">
         <v>28</v>
       </c>
-      <c r="D91" s="18">
+      <c r="D91" s="17">
         <f>0.35*gen!P91</f>
         <v>35.699999999999996</v>
       </c>
@@ -9503,7 +9559,7 @@
         <v>1</v>
       </c>
       <c r="G91">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-33.660000000000004</v>
       </c>
       <c r="H91">
@@ -9545,7 +9601,7 @@
       <c r="C92">
         <v>30</v>
       </c>
-      <c r="D92" s="18">
+      <c r="D92" s="17">
         <f>0.35*gen!P92</f>
         <v>28.874999999999996</v>
       </c>
@@ -9553,7 +9609,7 @@
         <v>1</v>
       </c>
       <c r="G92">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-27.225000000000001</v>
       </c>
       <c r="H92">
@@ -9595,7 +9651,7 @@
       <c r="C93">
         <v>8</v>
       </c>
-      <c r="D93" s="18">
+      <c r="D93" s="17">
         <f>0.35*gen!P93</f>
         <v>21.945</v>
       </c>
@@ -9603,7 +9659,7 @@
         <v>1</v>
       </c>
       <c r="G93">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-20.691000000000003</v>
       </c>
       <c r="H93">
@@ -9645,7 +9701,7 @@
       <c r="C94">
         <v>28</v>
       </c>
-      <c r="D94" s="18">
+      <c r="D94" s="17">
         <f>0.35*gen!P94</f>
         <v>17.639999999999997</v>
       </c>
@@ -9653,7 +9709,7 @@
         <v>1</v>
       </c>
       <c r="G94">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-16.632000000000001</v>
       </c>
       <c r="H94">
@@ -9695,7 +9751,7 @@
       <c r="C95">
         <v>29</v>
       </c>
-      <c r="D95" s="18">
+      <c r="D95" s="17">
         <f>0.35*gen!P95</f>
         <v>110.6</v>
       </c>
@@ -9703,7 +9759,7 @@
         <v>1</v>
       </c>
       <c r="G95">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-104.28</v>
       </c>
       <c r="H95">
@@ -9745,7 +9801,7 @@
       <c r="C96">
         <v>4</v>
       </c>
-      <c r="D96" s="18">
+      <c r="D96" s="17">
         <f>0.35*gen!P96</f>
         <v>29.4</v>
       </c>
@@ -9753,7 +9809,7 @@
         <v>1</v>
       </c>
       <c r="G96">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-27.720000000000002</v>
       </c>
       <c r="H96">
@@ -9795,7 +9851,7 @@
       <c r="C97">
         <v>4</v>
       </c>
-      <c r="D97" s="18">
+      <c r="D97" s="17">
         <f>0.35*gen!P97</f>
         <v>22.049999999999997</v>
       </c>
@@ -9803,7 +9859,7 @@
         <v>1</v>
       </c>
       <c r="G97">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-20.790000000000003</v>
       </c>
       <c r="H97">
@@ -9845,7 +9901,7 @@
       <c r="C98">
         <v>29</v>
       </c>
-      <c r="D98" s="18">
+      <c r="D98" s="17">
         <f>0.35*gen!P98</f>
         <v>273.7</v>
       </c>
@@ -9853,7 +9909,7 @@
         <v>1</v>
       </c>
       <c r="G98">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-258.06</v>
       </c>
       <c r="H98">
@@ -9895,7 +9951,7 @@
       <c r="C99">
         <v>32</v>
       </c>
-      <c r="D99" s="18">
+      <c r="D99" s="17">
         <f>0.35*gen!P99</f>
         <v>288.04999999999995</v>
       </c>
@@ -9903,7 +9959,7 @@
         <v>1</v>
       </c>
       <c r="G99">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-271.59000000000003</v>
       </c>
       <c r="H99">
@@ -9945,7 +10001,7 @@
       <c r="C100">
         <v>11</v>
       </c>
-      <c r="D100" s="18">
+      <c r="D100" s="17">
         <f>0.35*gen!P100</f>
         <v>234.14999999999998</v>
       </c>
@@ -9953,7 +10009,7 @@
         <v>1</v>
       </c>
       <c r="G100">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-220.77</v>
       </c>
       <c r="H100">
@@ -9995,7 +10051,7 @@
       <c r="C101">
         <v>25</v>
       </c>
-      <c r="D101" s="18">
+      <c r="D101" s="17">
         <f>0.35*gen!P101</f>
         <v>829.5</v>
       </c>
@@ -10003,7 +10059,7 @@
         <v>1</v>
       </c>
       <c r="G101">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-782.1</v>
       </c>
       <c r="H101">
@@ -10045,7 +10101,7 @@
       <c r="C102">
         <v>17</v>
       </c>
-      <c r="D102" s="18">
+      <c r="D102" s="17">
         <f>0.35*gen!P102</f>
         <v>94.85</v>
       </c>
@@ -10053,7 +10109,7 @@
         <v>1</v>
       </c>
       <c r="G102">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-89.43</v>
       </c>
       <c r="H102">
@@ -10095,7 +10151,7 @@
       <c r="C103">
         <v>6</v>
       </c>
-      <c r="D103" s="18">
+      <c r="D103" s="17">
         <f>0.35*gen!P103</f>
         <v>351.75</v>
       </c>
@@ -10103,7 +10159,7 @@
         <v>1</v>
       </c>
       <c r="G103">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-331.65000000000003</v>
       </c>
       <c r="H103">
@@ -10145,7 +10201,7 @@
       <c r="C104">
         <v>3</v>
       </c>
-      <c r="D104" s="18">
+      <c r="D104" s="17">
         <f>0.35*gen!P104</f>
         <v>236.95</v>
       </c>
@@ -10153,7 +10209,7 @@
         <v>1</v>
       </c>
       <c r="G104">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-223.41</v>
       </c>
       <c r="H104">
@@ -10195,7 +10251,7 @@
       <c r="C105">
         <v>9</v>
       </c>
-      <c r="D105" s="18">
+      <c r="D105" s="17">
         <f>0.35*gen!P105</f>
         <v>103.94999999999999</v>
       </c>
@@ -10203,7 +10259,7 @@
         <v>1</v>
       </c>
       <c r="G105">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-98.01</v>
       </c>
       <c r="H105">
@@ -10245,7 +10301,7 @@
       <c r="C106">
         <v>34</v>
       </c>
-      <c r="D106" s="18">
+      <c r="D106" s="17">
         <f>0.35*gen!P106</f>
         <v>33.25</v>
       </c>
@@ -10253,7 +10309,7 @@
         <v>1</v>
       </c>
       <c r="G106">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-31.35</v>
       </c>
       <c r="H106">
@@ -10295,7 +10351,7 @@
       <c r="C107">
         <v>26</v>
       </c>
-      <c r="D107" s="18">
+      <c r="D107" s="17">
         <f>0.35*gen!P107</f>
         <v>47.949999999999996</v>
       </c>
@@ -10303,7 +10359,7 @@
         <v>1</v>
       </c>
       <c r="G107">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-45.21</v>
       </c>
       <c r="H107">
@@ -10345,7 +10401,7 @@
       <c r="C108">
         <v>22</v>
       </c>
-      <c r="D108" s="18">
+      <c r="D108" s="17">
         <f>0.35*gen!P108</f>
         <v>162.75</v>
       </c>
@@ -10353,7 +10409,7 @@
         <v>1</v>
       </c>
       <c r="G108">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-153.45000000000002</v>
       </c>
       <c r="H108">
@@ -10395,7 +10451,7 @@
       <c r="C109">
         <v>10</v>
       </c>
-      <c r="D109" s="18">
+      <c r="D109" s="17">
         <f>0.35*gen!P109</f>
         <v>12.95</v>
       </c>
@@ -10403,7 +10459,7 @@
         <v>1</v>
       </c>
       <c r="G109">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-12.21</v>
       </c>
       <c r="H109">
@@ -10453,7 +10509,7 @@
         <v>1</v>
       </c>
       <c r="G110">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-36.300000000000004</v>
       </c>
       <c r="H110">
@@ -10503,7 +10559,7 @@
         <v>1</v>
       </c>
       <c r="G111">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-33.660000000000004</v>
       </c>
       <c r="H111">
@@ -10553,7 +10609,7 @@
         <v>1</v>
       </c>
       <c r="G112">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-21.12</v>
       </c>
       <c r="H112">
@@ -10603,7 +10659,7 @@
         <v>1</v>
       </c>
       <c r="G113">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-17.984999999999999</v>
       </c>
       <c r="H113">
@@ -10653,7 +10709,7 @@
         <v>1</v>
       </c>
       <c r="G114">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>-2382.6</v>
       </c>
       <c r="H114">
@@ -10703,7 +10759,7 @@
         <v>1</v>
       </c>
       <c r="G115">
-        <f t="shared" ref="G115:G146" si="8">-H115</f>
+        <f t="shared" ref="G115:G146" si="9">-H115</f>
         <v>-3065.3700000000003</v>
       </c>
       <c r="H115">
@@ -10753,7 +10809,7 @@
         <v>1</v>
       </c>
       <c r="G116">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1011.7800000000001</v>
       </c>
       <c r="H116">
@@ -10803,7 +10859,7 @@
         <v>1</v>
       </c>
       <c r="G117">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1165.56</v>
       </c>
       <c r="H117">
@@ -10853,7 +10909,7 @@
         <v>1</v>
       </c>
       <c r="G118">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-3480.84</v>
       </c>
       <c r="H118">
@@ -10903,7 +10959,7 @@
         <v>1</v>
       </c>
       <c r="G119">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1697.19</v>
       </c>
       <c r="H119">
@@ -10953,7 +11009,7 @@
         <v>1</v>
       </c>
       <c r="G120">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1293.27</v>
       </c>
       <c r="H120">
@@ -11003,7 +11059,7 @@
         <v>1</v>
       </c>
       <c r="G121">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1679.3700000000001</v>
       </c>
       <c r="H121">
@@ -11053,7 +11109,7 @@
         <v>1</v>
       </c>
       <c r="G122">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-2079.33</v>
       </c>
       <c r="H122">
@@ -11103,7 +11159,7 @@
         <v>1</v>
       </c>
       <c r="G123">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1959.8700000000001</v>
       </c>
       <c r="H123">
@@ -11153,7 +11209,7 @@
         <v>1</v>
       </c>
       <c r="G124">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-4302.87</v>
       </c>
       <c r="H124">
@@ -11203,7 +11259,7 @@
         <v>1</v>
       </c>
       <c r="G125">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1405.8</v>
       </c>
       <c r="H125">
@@ -11245,7 +11301,7 @@
       <c r="C126" s="10">
         <v>28</v>
       </c>
-      <c r="D126" s="18">
+      <c r="D126" s="17">
         <f>0.35*gen!P126</f>
         <v>266</v>
       </c>
@@ -11253,7 +11309,7 @@
         <v>1</v>
       </c>
       <c r="G126">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-250.8</v>
       </c>
       <c r="H126">
@@ -11295,7 +11351,7 @@
       <c r="C127" s="10">
         <v>28</v>
       </c>
-      <c r="D127" s="18">
+      <c r="D127" s="17">
         <f>0.35*gen!P127</f>
         <v>266</v>
       </c>
@@ -11303,7 +11359,7 @@
         <v>1</v>
       </c>
       <c r="G127">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-250.8</v>
       </c>
       <c r="H127">
@@ -11345,7 +11401,7 @@
       <c r="C128" s="10">
         <v>12</v>
       </c>
-      <c r="D128" s="18">
+      <c r="D128" s="17">
         <f>0.35*gen!P128</f>
         <v>265.64999999999998</v>
       </c>
@@ -11353,7 +11409,7 @@
         <v>1</v>
       </c>
       <c r="G128">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-250.47</v>
       </c>
       <c r="H128">
@@ -11395,7 +11451,7 @@
       <c r="C129" s="10">
         <v>12</v>
       </c>
-      <c r="D129" s="18">
+      <c r="D129" s="17">
         <f>0.35*gen!P129</f>
         <v>264.59999999999997</v>
       </c>
@@ -11403,7 +11459,7 @@
         <v>1</v>
       </c>
       <c r="G129">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-249.48000000000002</v>
       </c>
       <c r="H129">
@@ -11445,7 +11501,7 @@
       <c r="C130" s="10">
         <v>12</v>
       </c>
-      <c r="D130" s="18">
+      <c r="D130" s="17">
         <f>0.35*gen!P130</f>
         <v>244.99999999999997</v>
       </c>
@@ -11453,7 +11509,7 @@
         <v>1</v>
       </c>
       <c r="G130">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-231</v>
       </c>
       <c r="H130">
@@ -11495,7 +11551,7 @@
       <c r="C131" s="10">
         <v>12</v>
       </c>
-      <c r="D131" s="18">
+      <c r="D131" s="17">
         <f>0.35*gen!P131</f>
         <v>203</v>
       </c>
@@ -11503,7 +11559,7 @@
         <v>1</v>
       </c>
       <c r="G131">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-191.4</v>
       </c>
       <c r="H131">
@@ -11545,7 +11601,7 @@
       <c r="C132" s="10">
         <v>11</v>
       </c>
-      <c r="D132" s="18">
+      <c r="D132" s="17">
         <f>0.35*gen!P132</f>
         <v>263.2</v>
       </c>
@@ -11553,7 +11609,7 @@
         <v>1</v>
       </c>
       <c r="G132">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-248.16000000000003</v>
       </c>
       <c r="H132">
@@ -11595,7 +11651,7 @@
       <c r="C133" s="10">
         <v>11</v>
       </c>
-      <c r="D133" s="18">
+      <c r="D133" s="17">
         <f>0.35*gen!P133</f>
         <v>256.02499999999998</v>
       </c>
@@ -11603,7 +11659,7 @@
         <v>1</v>
       </c>
       <c r="G133">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-241.39500000000001</v>
       </c>
       <c r="H133">
@@ -11645,7 +11701,7 @@
       <c r="C134" s="10">
         <v>11</v>
       </c>
-      <c r="D134" s="18">
+      <c r="D134" s="17">
         <f>0.35*gen!P134</f>
         <v>6.6499999999999995</v>
       </c>
@@ -11653,7 +11709,7 @@
         <v>1</v>
       </c>
       <c r="G134">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-6.2700000000000005</v>
       </c>
       <c r="H134">
@@ -11695,7 +11751,7 @@
       <c r="C135" s="10">
         <v>28</v>
       </c>
-      <c r="D135" s="18">
+      <c r="D135" s="17">
         <f>0.35*gen!P135</f>
         <v>700</v>
       </c>
@@ -11703,7 +11759,7 @@
         <v>1</v>
       </c>
       <c r="G135">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-660</v>
       </c>
       <c r="H135">
@@ -11745,7 +11801,7 @@
       <c r="C136" s="10">
         <v>11</v>
       </c>
-      <c r="D136" s="18">
+      <c r="D136" s="17">
         <f>0.35*gen!P136</f>
         <v>700</v>
       </c>
@@ -11753,7 +11809,7 @@
         <v>1</v>
       </c>
       <c r="G136">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-660</v>
       </c>
       <c r="H136">
@@ -11795,7 +11851,7 @@
       <c r="C137" s="10">
         <v>28</v>
       </c>
-      <c r="D137" s="18">
+      <c r="D137" s="17">
         <f>0.35*gen!P137</f>
         <v>700</v>
       </c>
@@ -11803,7 +11859,7 @@
         <v>1</v>
       </c>
       <c r="G137">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-660</v>
       </c>
       <c r="H137">
@@ -11845,7 +11901,7 @@
       <c r="C138" s="10">
         <v>22</v>
       </c>
-      <c r="D138" s="18">
+      <c r="D138" s="17">
         <f>0.35*gen!P138</f>
         <v>1050</v>
       </c>
@@ -11853,7 +11909,7 @@
         <v>1</v>
       </c>
       <c r="G138">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-990</v>
       </c>
       <c r="H138">
@@ -11895,7 +11951,7 @@
       <c r="C139" s="10">
         <v>22</v>
       </c>
-      <c r="D139" s="18">
+      <c r="D139" s="17">
         <f>0.35*gen!P139</f>
         <v>1050</v>
       </c>
@@ -11903,7 +11959,7 @@
         <v>1</v>
       </c>
       <c r="G139">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-990</v>
       </c>
       <c r="H139">
@@ -11945,7 +12001,7 @@
       <c r="C140" s="10">
         <v>21</v>
       </c>
-      <c r="D140" s="18">
+      <c r="D140" s="17">
         <f>0.35*gen!P140</f>
         <v>1400</v>
       </c>
@@ -11953,7 +12009,7 @@
         <v>1</v>
       </c>
       <c r="G140">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-1320</v>
       </c>
       <c r="H140">
@@ -11995,7 +12051,7 @@
       <c r="C141" s="10">
         <v>51</v>
       </c>
-      <c r="D141" s="18">
+      <c r="D141" s="17">
         <f>0.35*gen!P141</f>
         <v>28</v>
       </c>
@@ -12003,7 +12059,7 @@
         <v>1</v>
       </c>
       <c r="G141">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-26.400000000000002</v>
       </c>
       <c r="H141">
@@ -12045,7 +12101,7 @@
       <c r="C142" s="10">
         <v>25</v>
       </c>
-      <c r="D142" s="18">
+      <c r="D142" s="17">
         <f>0.35*gen!P142</f>
         <v>21</v>
       </c>
@@ -12053,7 +12109,7 @@
         <v>1</v>
       </c>
       <c r="G142">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-19.8</v>
       </c>
       <c r="H142">
@@ -12095,7 +12151,7 @@
       <c r="C143" s="10">
         <v>47</v>
       </c>
-      <c r="D143" s="18">
+      <c r="D143" s="17">
         <f>0.35*gen!P143</f>
         <v>17.5</v>
       </c>
@@ -12103,7 +12159,7 @@
         <v>1</v>
       </c>
       <c r="G143">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-16.5</v>
       </c>
       <c r="H143">
@@ -12153,7 +12209,7 @@
         <v>1</v>
       </c>
       <c r="G144">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-29.37</v>
       </c>
       <c r="H144">
@@ -12203,7 +12259,7 @@
         <v>1</v>
       </c>
       <c r="G145">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-18.150000000000002</v>
       </c>
       <c r="H145">
@@ -12253,7 +12309,7 @@
         <v>1</v>
       </c>
       <c r="G146">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-48.84</v>
       </c>
       <c r="H146">
@@ -12303,7 +12359,7 @@
         <v>1</v>
       </c>
       <c r="G147">
-        <f t="shared" ref="G147:G178" si="9">-H147</f>
+        <f t="shared" ref="G147:G171" si="10">-H147</f>
         <v>-16.5</v>
       </c>
       <c r="H147">
@@ -12353,7 +12409,7 @@
         <v>1</v>
       </c>
       <c r="G148">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-26.400000000000002</v>
       </c>
       <c r="H148">
@@ -12403,7 +12459,7 @@
         <v>1</v>
       </c>
       <c r="G149">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-20.130000000000003</v>
       </c>
       <c r="H149">
@@ -12453,7 +12509,7 @@
         <v>1</v>
       </c>
       <c r="G150">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-24.42</v>
       </c>
       <c r="H150">
@@ -12503,7 +12559,7 @@
         <v>1</v>
       </c>
       <c r="G151">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-18.150000000000002</v>
       </c>
       <c r="H151">
@@ -12553,7 +12609,7 @@
         <v>1</v>
       </c>
       <c r="G152">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-18.150000000000002</v>
       </c>
       <c r="H152">
@@ -12603,7 +12659,7 @@
         <v>1</v>
       </c>
       <c r="G153">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-24.75</v>
       </c>
       <c r="H153">
@@ -12653,7 +12709,7 @@
         <v>1</v>
       </c>
       <c r="G154">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-17.82</v>
       </c>
       <c r="H154">
@@ -12703,7 +12759,7 @@
         <v>1</v>
       </c>
       <c r="G155">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-21.45</v>
       </c>
       <c r="H155">
@@ -12753,7 +12809,7 @@
         <v>1</v>
       </c>
       <c r="G156">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-20.46</v>
       </c>
       <c r="H156">
@@ -12803,7 +12859,7 @@
         <v>1</v>
       </c>
       <c r="G157">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-31.020000000000003</v>
       </c>
       <c r="H157">
@@ -12853,7 +12909,7 @@
         <v>1</v>
       </c>
       <c r="G158">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-31.68</v>
       </c>
       <c r="H158">
@@ -12903,7 +12959,7 @@
         <v>1</v>
       </c>
       <c r="G159">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-28.380000000000003</v>
       </c>
       <c r="H159">
@@ -12953,7 +13009,7 @@
         <v>1</v>
       </c>
       <c r="G160">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-43.56</v>
       </c>
       <c r="H160">
@@ -13003,7 +13059,7 @@
         <v>1</v>
       </c>
       <c r="G161">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-21.45</v>
       </c>
       <c r="H161">
@@ -13053,7 +13109,7 @@
         <v>1</v>
       </c>
       <c r="G162">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-38.28</v>
       </c>
       <c r="H162">
@@ -13103,7 +13159,7 @@
         <v>1</v>
       </c>
       <c r="G163">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-20.790000000000003</v>
       </c>
       <c r="H163">
@@ -13153,7 +13209,7 @@
         <v>1</v>
       </c>
       <c r="G164">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-19.14</v>
       </c>
       <c r="H164">
@@ -13203,7 +13259,7 @@
         <v>1</v>
       </c>
       <c r="G165">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-37.950000000000003</v>
       </c>
       <c r="H165">
@@ -13253,7 +13309,7 @@
         <v>1</v>
       </c>
       <c r="G166">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-35.64</v>
       </c>
       <c r="H166">
@@ -13303,7 +13359,7 @@
         <v>1</v>
       </c>
       <c r="G167">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-17.490000000000002</v>
       </c>
       <c r="H167">
@@ -13353,7 +13409,7 @@
         <v>1</v>
       </c>
       <c r="G168">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-19.14</v>
       </c>
       <c r="H168">
@@ -13403,7 +13459,7 @@
         <v>1</v>
       </c>
       <c r="G169">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-20.46</v>
       </c>
       <c r="H169">
@@ -13453,7 +13509,7 @@
         <v>1</v>
       </c>
       <c r="G170">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-44.88</v>
       </c>
       <c r="H170">
@@ -13503,7 +13559,7 @@
         <v>1</v>
       </c>
       <c r="G171">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-19.470000000000002</v>
       </c>
       <c r="H171">
@@ -13606,13 +13662,14 @@
         <v>1</v>
       </c>
       <c r="H2" s="16">
-        <v>100</v>
+        <f>0.24*2000</f>
+        <v>480</v>
       </c>
       <c r="I2">
-        <v>-1972</v>
+        <v>-2340</v>
       </c>
       <c r="J2">
-        <v>1972</v>
+        <v>2340</v>
       </c>
       <c r="K2">
         <v>-5000</v>
@@ -17554,10 +17611,10 @@
       <c r="A83" s="4">
         <v>81</v>
       </c>
-      <c r="B83" s="20" t="s">
+      <c r="B83" s="19" t="s">
         <v>463</v>
       </c>
-      <c r="D83" s="20">
+      <c r="D83" s="19">
         <v>30</v>
       </c>
       <c r="E83">
@@ -17601,10 +17658,10 @@
       <c r="A84" s="4">
         <v>82</v>
       </c>
-      <c r="B84" s="20" t="s">
+      <c r="B84" s="19" t="s">
         <v>464</v>
       </c>
-      <c r="D84" s="20">
+      <c r="D84" s="19">
         <v>30</v>
       </c>
       <c r="E84">
@@ -17648,13 +17705,13 @@
       <c r="A85" s="4">
         <v>83</v>
       </c>
-      <c r="B85" s="20" t="s">
+      <c r="B85" s="19" t="s">
         <v>465</v>
       </c>
       <c r="D85">
         <v>22</v>
       </c>
-      <c r="E85" s="20">
+      <c r="E85" s="19">
         <v>50</v>
       </c>
       <c r="F85" s="8">
@@ -17695,13 +17752,13 @@
       <c r="A86" s="4">
         <v>84</v>
       </c>
-      <c r="B86" s="20" t="s">
+      <c r="B86" s="19" t="s">
         <v>466</v>
       </c>
       <c r="D86">
         <v>22</v>
       </c>
-      <c r="E86" s="20">
+      <c r="E86" s="19">
         <v>50</v>
       </c>
       <c r="F86" s="8">
@@ -17742,7 +17799,7 @@
       <c r="A87" s="4">
         <v>85</v>
       </c>
-      <c r="B87" s="20" t="s">
+      <c r="B87" s="19" t="s">
         <v>271</v>
       </c>
       <c r="D87">
@@ -17789,7 +17846,7 @@
       <c r="A88" s="4">
         <v>86</v>
       </c>
-      <c r="B88" s="20" t="s">
+      <c r="B88" s="19" t="s">
         <v>272</v>
       </c>
       <c r="D88">

</xml_diff>